<commit_message>
Sonbol Salla subscription: confirmed cancelled, no revenue
Dar Sonbol subscribed on 20 Aug without the SPNS75 coupon applying, so it
charged full price (3,999.00 ex-VAT). They contacted Salla, the subscription
was cancelled, and they will re-subscribe with the discount.

Revenue stays 0.00 for this record — correct, since no money was retained.
Expect ~999.75 ex-VAT to appear once the discounted subscription is placed;
the weekly run will pick it up.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bb5MYX3TP7gHh1Nbcy8kyQ
</commit_message>
<xml_diff>
--- a/revenue-view/output/Nasam_Revenue_View.xlsx
+++ b/revenue-view/output/Nasam_Revenue_View.xlsx
@@ -14686,12 +14686,12 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>— (full price)</t>
+          <t>none — coupon missed</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>CANCELLED — confirm paid/refunded</t>
+          <t>Cancelled via Salla — re-subscribing with SPNS75</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Weekly run 3 (6 Sep): Wafeq refreshed, drafts excluded from billed with memo row
- Wafeq API snapshot 6 Sep: 164 invoices; four August monthly invoices drafted 31 Aug (12,013.72) now shown as a memo line and excluded from billed; five invoices moved to PAID
- Platform sales/POs not refreshed (read layer unavailable); carried from 30 Aug
- Verification: 120 client-month cells 0 mismatches, 220 nested cells 0 mismatches, allocation OK, TOTAL identity holds

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bb5MYX3TP7gHh1Nbcy8kyQ
</commit_message>
<xml_diff>
--- a/revenue-view/output/Nasam_Revenue_View.xlsx
+++ b/revenue-view/output/Nasam_Revenue_View.xlsx
@@ -491,7 +491,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Nasam Revenue View — weekly run · 23 Aug 2026</t>
+          <t>Nasam Revenue View — weekly run · 6 Sep 2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -504,7 +504,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>First automated Sunday run. Billing source switched to the WAFEQ API (reconciled against the 17-Aug manual export before switching). Retail reads closed POs directly from the platform (values live since 20 Aug), netted against retail invoices already raised in Wafeq. Sonbol was renamed in the platform ('Sonbol') and its from-integration sales refreshed.</t>
+          <t>Third automated Sunday run. Wafeq pulled via API on 6 Sep (164 invoices): no new invoices issued since 30 Aug; four August monthly invoices are drafted (31 Aug, 12,013.72) and enter billed once sent; five invoices moved to PAID (Alfaris May–Jul, Inivita Jul, INV-000151). The platform read layer was unavailable this run, so platform sales, purchase orders and Sonbol's from-integration figure are carried from the 30 Aug pull (August through 30 Aug; no September GMV yet). The six duplicated Alfaris retail invoices (INV-000169/170/171/181/182/183, 739.48) are still SENT in Wafeq with no credit note, so the Dec–Feb over-billing is still shown.</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Wafeq API snapshot 23 Aug (160 invoices) · platform revenue + purchase orders pulled 23 Aug · churned-brand snapshots 15 Aug (the read layer does not serve deactivated brands) · Salla Partners export 18 Aug (manual) · rate card 17 Aug.</t>
+          <t>Wafeq API snapshot 6 Sep (164 invoices) · platform revenue + purchase orders pulled 30 Aug (not refreshed this run) · churned-brand snapshots 15 Aug (the read layer does not serve deactivated brands) · Salla Partners export 30 Aug (manual, 26 records) · rate card 17 Aug.</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N121"/>
+  <dimension ref="A1:N122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4108,7 +4108,7 @@
     <row r="100">
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Retail commission — closed POs, to invoice</t>
+          <t>Memo: drafted in Wafeq, not yet issued (not in billed)</t>
         </is>
       </c>
       <c r="C100" s="5" t="n"/>
@@ -4121,21 +4121,21 @@
       <c r="J100" s="5" t="n"/>
       <c r="K100" s="5" t="n"/>
       <c r="L100" s="5" t="n">
-        <v>17.14</v>
+        <v>12013.72</v>
       </c>
       <c r="M100" s="5" t="n">
-        <v>17.14</v>
+        <v>12013.72</v>
       </c>
       <c r="N100" s="3" t="inlineStr">
         <is>
-          <t>Nasam platform — closed POs — net of retail already billed in Wafeq</t>
+          <t>Wafeq invoice export — DRAFT status; enters billed once sent</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>SaaS subscriptions (Salla App Store, gross)</t>
+          <t>Retail commission — closed POs, to invoice</t>
         </is>
       </c>
       <c r="C101" s="5" t="n"/>
@@ -4144,29 +4144,25 @@
       <c r="F101" s="5" t="n"/>
       <c r="G101" s="5" t="n"/>
       <c r="H101" s="5" t="n"/>
-      <c r="I101" s="5" t="n">
-        <v>999.75</v>
-      </c>
+      <c r="I101" s="5" t="n"/>
       <c r="J101" s="5" t="n"/>
-      <c r="K101" s="5" t="n">
-        <v>449</v>
-      </c>
+      <c r="K101" s="5" t="n"/>
       <c r="L101" s="5" t="n">
-        <v>999.75</v>
+        <v>17.14</v>
       </c>
       <c r="M101" s="5" t="n">
-        <v>2448.5</v>
+        <v>17.14</v>
       </c>
       <c r="N101" s="3" t="inlineStr">
         <is>
-          <t>Salla Partners export</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" outlineLevel="1">
+          <t>Nasam platform — closed POs — net of retail already billed in Wafeq</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    محمصة نقوش (Nokush) — annual, paid May 2026</t>
+          <t>SaaS subscriptions (Salla App Store, gross)</t>
         </is>
       </c>
       <c r="C102" s="5" t="n"/>
@@ -4179,10 +4175,14 @@
         <v>999.75</v>
       </c>
       <c r="J102" s="5" t="n"/>
-      <c r="K102" s="5" t="n"/>
-      <c r="L102" s="5" t="n"/>
+      <c r="K102" s="5" t="n">
+        <v>449</v>
+      </c>
+      <c r="L102" s="5" t="n">
+        <v>999.75</v>
+      </c>
       <c r="M102" s="5" t="n">
-        <v>999.75</v>
+        <v>2448.5</v>
       </c>
       <c r="N102" s="3" t="inlineStr">
         <is>
@@ -4193,7 +4193,7 @@
     <row r="103" outlineLevel="1">
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    SONDOS — monthly, paid Jul 2026</t>
+          <t xml:space="preserve">    محمصة نقوش (Nokush) — annual, paid May 2026</t>
         </is>
       </c>
       <c r="C103" s="5" t="n"/>
@@ -4202,14 +4202,14 @@
       <c r="F103" s="5" t="n"/>
       <c r="G103" s="5" t="n"/>
       <c r="H103" s="5" t="n"/>
-      <c r="I103" s="5" t="n"/>
+      <c r="I103" s="5" t="n">
+        <v>999.75</v>
+      </c>
       <c r="J103" s="5" t="n"/>
-      <c r="K103" s="5" t="n">
-        <v>449</v>
-      </c>
+      <c r="K103" s="5" t="n"/>
       <c r="L103" s="5" t="n"/>
       <c r="M103" s="5" t="n">
-        <v>449</v>
+        <v>999.75</v>
       </c>
       <c r="N103" s="3" t="inlineStr">
         <is>
@@ -4220,7 +4220,7 @@
     <row r="104" outlineLevel="1">
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    SONDOS — annual, paid Aug 2026</t>
+          <t xml:space="preserve">    SONDOS — monthly, paid Jul 2026</t>
         </is>
       </c>
       <c r="C104" s="5" t="n"/>
@@ -4231,12 +4231,12 @@
       <c r="H104" s="5" t="n"/>
       <c r="I104" s="5" t="n"/>
       <c r="J104" s="5" t="n"/>
-      <c r="K104" s="5" t="n"/>
-      <c r="L104" s="5" t="n">
-        <v>999.75</v>
-      </c>
+      <c r="K104" s="5" t="n">
+        <v>449</v>
+      </c>
+      <c r="L104" s="5" t="n"/>
       <c r="M104" s="5" t="n">
-        <v>999.75</v>
+        <v>449</v>
       </c>
       <c r="N104" s="3" t="inlineStr">
         <is>
@@ -4244,10 +4244,10 @@
         </is>
       </c>
     </row>
-    <row r="105">
+    <row r="105" outlineLevel="1">
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>less: Salla share (15%)</t>
+          <t xml:space="preserve">    SONDOS — annual, paid Aug 2026</t>
         </is>
       </c>
       <c r="C105" s="5" t="n"/>
@@ -4256,158 +4256,142 @@
       <c r="F105" s="5" t="n"/>
       <c r="G105" s="5" t="n"/>
       <c r="H105" s="5" t="n"/>
-      <c r="I105" s="5" t="n">
+      <c r="I105" s="5" t="n"/>
+      <c r="J105" s="5" t="n"/>
+      <c r="K105" s="5" t="n"/>
+      <c r="L105" s="5" t="n">
+        <v>999.75</v>
+      </c>
+      <c r="M105" s="5" t="n">
+        <v>999.75</v>
+      </c>
+      <c r="N105" s="3" t="inlineStr">
+        <is>
+          <t>Salla Partners export</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>less: Salla share (15%)</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="n"/>
+      <c r="D106" s="5" t="n"/>
+      <c r="E106" s="5" t="n"/>
+      <c r="F106" s="5" t="n"/>
+      <c r="G106" s="5" t="n"/>
+      <c r="H106" s="5" t="n"/>
+      <c r="I106" s="5" t="n">
         <v>-149.96</v>
       </c>
-      <c r="J105" s="5" t="n"/>
-      <c r="K105" s="5" t="n">
+      <c r="J106" s="5" t="n"/>
+      <c r="K106" s="5" t="n">
         <v>-67.34999999999999</v>
       </c>
-      <c r="L105" s="5" t="n">
+      <c r="L106" s="5" t="n">
         <v>-149.96</v>
       </c>
-      <c r="M105" s="5" t="n">
+      <c r="M106" s="5" t="n">
         <v>-367.27</v>
       </c>
-      <c r="N105" s="3" t="inlineStr">
+      <c r="N106" s="3" t="inlineStr">
         <is>
           <t>15% per Tarik — not pullable from Salla</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="B106" s="6" t="inlineStr">
+    <row r="107">
+      <c r="B107" s="6" t="inlineStr">
         <is>
           <t>TOTAL REVENUE</t>
         </is>
       </c>
-      <c r="C106" s="7" t="n">
+      <c r="C107" s="7" t="n">
         <v>31390.44</v>
       </c>
-      <c r="D106" s="7" t="n">
+      <c r="D107" s="7" t="n">
         <v>21947.73</v>
       </c>
-      <c r="E106" s="7" t="n">
+      <c r="E107" s="7" t="n">
         <v>26212.8</v>
       </c>
-      <c r="F106" s="7" t="n">
+      <c r="F107" s="7" t="n">
         <v>19517.67</v>
       </c>
-      <c r="G106" s="7" t="n">
+      <c r="G107" s="7" t="n">
         <v>27125.53</v>
       </c>
-      <c r="H106" s="7" t="n">
+      <c r="H107" s="7" t="n">
         <v>27486.22</v>
       </c>
-      <c r="I106" s="7" t="n">
+      <c r="I107" s="7" t="n">
         <v>22806.22</v>
       </c>
-      <c r="J106" s="7" t="n">
+      <c r="J107" s="7" t="n">
         <v>16243.45</v>
       </c>
-      <c r="K106" s="7" t="n">
+      <c r="K107" s="7" t="n">
         <v>7680.6</v>
       </c>
-      <c r="L106" s="7" t="n">
+      <c r="L107" s="7" t="n">
         <v>3547.81</v>
       </c>
-      <c r="M106" s="7" t="n">
+      <c r="M107" s="7" t="n">
         <v>203958.46</v>
       </c>
-      <c r="N106" s="3" t="inlineStr">
+      <c r="N107" s="3" t="inlineStr">
         <is>
           <t>Billed + to-invoice + SaaS net of Salla share</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="B108" s="1" t="inlineStr">
+    <row r="109">
+      <c r="B109" s="1" t="inlineStr">
         <is>
           <t>BY CLIENT (billed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>Alfaris Group</t>
-        </is>
-      </c>
-      <c r="C109" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D109" s="5" t="n">
-        <v>2717.44</v>
-      </c>
-      <c r="E109" s="5" t="n">
-        <v>5230.11</v>
-      </c>
-      <c r="F109" s="5" t="n">
-        <v>3123.95</v>
-      </c>
-      <c r="G109" s="5" t="n">
-        <v>2640.55</v>
-      </c>
-      <c r="H109" s="5" t="n">
-        <v>2840.27</v>
-      </c>
-      <c r="I109" s="5" t="n">
-        <v>4081.37</v>
-      </c>
-      <c r="J109" s="5" t="n">
-        <v>3921.48</v>
-      </c>
-      <c r="K109" s="5" t="n">
-        <v>3290.53</v>
-      </c>
-      <c r="L109" s="5" t="n">
-        <v>2513.78</v>
-      </c>
-      <c r="M109" s="5" t="n">
-        <v>32859.48</v>
-      </c>
-      <c r="N109" s="3" t="inlineStr">
-        <is>
-          <t>Wafeq invoice export</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Inivita</t>
+          <t>Alfaris Group</t>
         </is>
       </c>
       <c r="C110" s="5" t="n">
-        <v>3269.61</v>
+        <v>2500</v>
       </c>
       <c r="D110" s="5" t="n">
-        <v>3598.8</v>
+        <v>2717.44</v>
       </c>
       <c r="E110" s="5" t="n">
-        <v>3591.47</v>
+        <v>5230.11</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>4252.12</v>
+        <v>3123.95</v>
       </c>
       <c r="G110" s="5" t="n">
-        <v>3792.64</v>
+        <v>2640.55</v>
       </c>
       <c r="H110" s="5" t="n">
-        <v>3047.98</v>
+        <v>2840.27</v>
       </c>
       <c r="I110" s="5" t="n">
-        <v>3218.29</v>
+        <v>4081.37</v>
       </c>
       <c r="J110" s="5" t="n">
-        <v>2377.85</v>
+        <v>3921.48</v>
       </c>
       <c r="K110" s="5" t="n">
-        <v>2884.13</v>
-      </c>
-      <c r="L110" s="5" t="n"/>
+        <v>3290.53</v>
+      </c>
+      <c r="L110" s="5" t="n">
+        <v>2513.78</v>
+      </c>
       <c r="M110" s="5" t="n">
-        <v>30032.89</v>
+        <v>32859.48</v>
       </c>
       <c r="N110" s="3" t="inlineStr">
         <is>
@@ -4418,39 +4402,39 @@
     <row r="111">
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Nokush</t>
+          <t>Inivita</t>
         </is>
       </c>
       <c r="C111" s="5" t="n">
-        <v>338.91</v>
+        <v>3269.61</v>
       </c>
       <c r="D111" s="5" t="n">
-        <v>238.59</v>
+        <v>3598.8</v>
       </c>
       <c r="E111" s="5" t="n">
-        <v>180.02</v>
+        <v>3591.47</v>
       </c>
       <c r="F111" s="5" t="n">
-        <v>409.44</v>
+        <v>4252.12</v>
       </c>
       <c r="G111" s="5" t="n">
-        <v>326.25</v>
+        <v>3792.64</v>
       </c>
       <c r="H111" s="5" t="n">
-        <v>420.69</v>
+        <v>3047.98</v>
       </c>
       <c r="I111" s="5" t="n">
-        <v>655.84</v>
+        <v>3218.29</v>
       </c>
       <c r="J111" s="5" t="n">
-        <v>423.72</v>
+        <v>2377.85</v>
       </c>
       <c r="K111" s="5" t="n">
-        <v>319.26</v>
+        <v>2884.13</v>
       </c>
       <c r="L111" s="5" t="n"/>
       <c r="M111" s="5" t="n">
-        <v>3312.72</v>
+        <v>30032.89</v>
       </c>
       <c r="N111" s="3" t="inlineStr">
         <is>
@@ -4461,33 +4445,39 @@
     <row r="112">
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Wadi Halfa</t>
-        </is>
-      </c>
-      <c r="C112" s="5" t="n"/>
-      <c r="D112" s="5" t="n"/>
-      <c r="E112" s="5" t="n"/>
-      <c r="F112" s="5" t="n"/>
+          <t>Nokush</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="n">
+        <v>338.91</v>
+      </c>
+      <c r="D112" s="5" t="n">
+        <v>238.59</v>
+      </c>
+      <c r="E112" s="5" t="n">
+        <v>180.02</v>
+      </c>
+      <c r="F112" s="5" t="n">
+        <v>409.44</v>
+      </c>
       <c r="G112" s="5" t="n">
-        <v>3290.32</v>
+        <v>326.25</v>
       </c>
       <c r="H112" s="5" t="n">
-        <v>8.960000000000001</v>
+        <v>420.69</v>
       </c>
       <c r="I112" s="5" t="n">
-        <v>2024.04</v>
+        <v>655.84</v>
       </c>
       <c r="J112" s="5" t="n">
-        <v>2016.48</v>
+        <v>423.72</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>805.03</v>
-      </c>
-      <c r="L112" s="5" t="n">
-        <v>167.1</v>
-      </c>
+        <v>319.26</v>
+      </c>
+      <c r="L112" s="5" t="n"/>
       <c r="M112" s="5" t="n">
-        <v>8311.93</v>
+        <v>3312.72</v>
       </c>
       <c r="N112" s="3" t="inlineStr">
         <is>
@@ -4498,23 +4488,33 @@
     <row r="113">
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Dar Sonbol</t>
+          <t>Wadi Halfa</t>
         </is>
       </c>
       <c r="C113" s="5" t="n"/>
       <c r="D113" s="5" t="n"/>
       <c r="E113" s="5" t="n"/>
       <c r="F113" s="5" t="n"/>
-      <c r="G113" s="5" t="n"/>
-      <c r="H113" s="5" t="n"/>
-      <c r="I113" s="5" t="n"/>
+      <c r="G113" s="5" t="n">
+        <v>3290.32</v>
+      </c>
+      <c r="H113" s="5" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="I113" s="5" t="n">
+        <v>2024.04</v>
+      </c>
       <c r="J113" s="5" t="n">
-        <v>4000</v>
-      </c>
-      <c r="K113" s="5" t="n"/>
-      <c r="L113" s="5" t="n"/>
+        <v>2016.48</v>
+      </c>
+      <c r="K113" s="5" t="n">
+        <v>805.03</v>
+      </c>
+      <c r="L113" s="5" t="n">
+        <v>167.1</v>
+      </c>
       <c r="M113" s="5" t="n">
-        <v>4000</v>
+        <v>8311.93</v>
       </c>
       <c r="N113" s="3" t="inlineStr">
         <is>
@@ -4525,35 +4525,23 @@
     <row r="114">
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Two United  (churned 2026-05)</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D114" s="5" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E114" s="5" t="n">
-        <v>3606.59</v>
-      </c>
-      <c r="F114" s="5" t="n">
-        <v>2747.96</v>
-      </c>
-      <c r="G114" s="5" t="n">
-        <v>5631.76</v>
-      </c>
-      <c r="H114" s="5" t="n">
-        <v>5324.76</v>
-      </c>
-      <c r="I114" s="5" t="n">
-        <v>5462.25</v>
-      </c>
-      <c r="J114" s="5" t="n"/>
+          <t>Dar Sonbol</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="n"/>
+      <c r="D114" s="5" t="n"/>
+      <c r="E114" s="5" t="n"/>
+      <c r="F114" s="5" t="n"/>
+      <c r="G114" s="5" t="n"/>
+      <c r="H114" s="5" t="n"/>
+      <c r="I114" s="5" t="n"/>
+      <c r="J114" s="5" t="n">
+        <v>4000</v>
+      </c>
       <c r="K114" s="5" t="n"/>
       <c r="L114" s="5" t="n"/>
       <c r="M114" s="5" t="n">
-        <v>32773.32</v>
+        <v>4000</v>
       </c>
       <c r="N114" s="3" t="inlineStr">
         <is>
@@ -4564,37 +4552,35 @@
     <row r="115">
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Rimath  (churned 2026-06)</t>
+          <t>Two United  (churned 2026-05)</t>
         </is>
       </c>
       <c r="C115" s="5" t="n">
-        <v>3743.36</v>
+        <v>5000</v>
       </c>
       <c r="D115" s="5" t="n">
-        <v>2998.75</v>
+        <v>5000</v>
       </c>
       <c r="E115" s="5" t="n">
-        <v>3561.57</v>
+        <v>3606.59</v>
       </c>
       <c r="F115" s="5" t="n">
-        <v>4753.24</v>
+        <v>2747.96</v>
       </c>
       <c r="G115" s="5" t="n">
-        <v>3970.51</v>
+        <v>5631.76</v>
       </c>
       <c r="H115" s="5" t="n">
-        <v>3649.59</v>
+        <v>5324.76</v>
       </c>
       <c r="I115" s="5" t="n">
-        <v>3044.62</v>
-      </c>
-      <c r="J115" s="5" t="n">
-        <v>2819.43</v>
-      </c>
+        <v>5462.25</v>
+      </c>
+      <c r="J115" s="5" t="n"/>
       <c r="K115" s="5" t="n"/>
       <c r="L115" s="5" t="n"/>
       <c r="M115" s="5" t="n">
-        <v>28541.07</v>
+        <v>32773.32</v>
       </c>
       <c r="N115" s="3" t="inlineStr">
         <is>
@@ -4605,35 +4591,37 @@
     <row r="116">
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Ancy &amp; Shaya  (churned 2026-05)</t>
+          <t>Rimath  (churned 2026-06)</t>
         </is>
       </c>
       <c r="C116" s="5" t="n">
-        <v>3041.76</v>
+        <v>3743.36</v>
       </c>
       <c r="D116" s="5" t="n">
-        <v>2097.12</v>
+        <v>2998.75</v>
       </c>
       <c r="E116" s="5" t="n">
-        <v>2292.39</v>
+        <v>3561.57</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>2880.71</v>
+        <v>4753.24</v>
       </c>
       <c r="G116" s="5" t="n">
-        <v>2981.2</v>
+        <v>3970.51</v>
       </c>
       <c r="H116" s="5" t="n">
-        <v>2360.37</v>
+        <v>3649.59</v>
       </c>
       <c r="I116" s="5" t="n">
-        <v>1670.7</v>
-      </c>
-      <c r="J116" s="5" t="n"/>
+        <v>3044.62</v>
+      </c>
+      <c r="J116" s="5" t="n">
+        <v>2819.43</v>
+      </c>
       <c r="K116" s="5" t="n"/>
       <c r="L116" s="5" t="n"/>
       <c r="M116" s="5" t="n">
-        <v>17324.25</v>
+        <v>28541.07</v>
       </c>
       <c r="N116" s="3" t="inlineStr">
         <is>
@@ -4644,29 +4632,35 @@
     <row r="117">
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Gamesir  (churned 2026-02)</t>
+          <t>Ancy &amp; Shaya  (churned 2026-05)</t>
         </is>
       </c>
       <c r="C117" s="5" t="n">
-        <v>3161.37</v>
+        <v>3041.76</v>
       </c>
       <c r="D117" s="5" t="n">
-        <v>2732.77</v>
+        <v>2097.12</v>
       </c>
       <c r="E117" s="5" t="n">
-        <v>5143.07</v>
+        <v>2292.39</v>
       </c>
       <c r="F117" s="5" t="n">
-        <v>512.96</v>
-      </c>
-      <c r="G117" s="5" t="n"/>
-      <c r="H117" s="5" t="n"/>
-      <c r="I117" s="5" t="n"/>
+        <v>2880.71</v>
+      </c>
+      <c r="G117" s="5" t="n">
+        <v>2981.2</v>
+      </c>
+      <c r="H117" s="5" t="n">
+        <v>2360.37</v>
+      </c>
+      <c r="I117" s="5" t="n">
+        <v>1670.7</v>
+      </c>
       <c r="J117" s="5" t="n"/>
       <c r="K117" s="5" t="n"/>
       <c r="L117" s="5" t="n"/>
       <c r="M117" s="5" t="n">
-        <v>11550.17</v>
+        <v>17324.25</v>
       </c>
       <c r="N117" s="3" t="inlineStr">
         <is>
@@ -4677,20 +4671,20 @@
     <row r="118">
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Safwat Aljouf  (churned 2026-02)</t>
+          <t>Gamesir  (churned 2026-02)</t>
         </is>
       </c>
       <c r="C118" s="5" t="n">
-        <v>3585.43</v>
+        <v>3161.37</v>
       </c>
       <c r="D118" s="5" t="n">
-        <v>2564.26</v>
+        <v>2732.77</v>
       </c>
       <c r="E118" s="5" t="n">
-        <v>2607.58</v>
+        <v>5143.07</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>837.29</v>
+        <v>512.96</v>
       </c>
       <c r="G118" s="5" t="n"/>
       <c r="H118" s="5" t="n"/>
@@ -4699,7 +4693,7 @@
       <c r="K118" s="5" t="n"/>
       <c r="L118" s="5" t="n"/>
       <c r="M118" s="5" t="n">
-        <v>9594.559999999999</v>
+        <v>11550.17</v>
       </c>
       <c r="N118" s="3" t="inlineStr">
         <is>
@@ -4710,29 +4704,29 @@
     <row r="119">
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Reetal  (churned 2026-06)</t>
-        </is>
-      </c>
-      <c r="C119" s="5" t="n"/>
-      <c r="D119" s="5" t="n"/>
-      <c r="E119" s="5" t="n"/>
-      <c r="F119" s="5" t="n"/>
-      <c r="G119" s="5" t="n">
-        <v>4492.3</v>
-      </c>
-      <c r="H119" s="5" t="n">
-        <v>1033.1</v>
-      </c>
-      <c r="I119" s="5" t="n">
-        <v>1799.32</v>
-      </c>
-      <c r="J119" s="5" t="n">
-        <v>684.49</v>
-      </c>
+          <t>Safwat Aljouf  (churned 2026-02)</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="n">
+        <v>3585.43</v>
+      </c>
+      <c r="D119" s="5" t="n">
+        <v>2564.26</v>
+      </c>
+      <c r="E119" s="5" t="n">
+        <v>2607.58</v>
+      </c>
+      <c r="F119" s="5" t="n">
+        <v>837.29</v>
+      </c>
+      <c r="G119" s="5" t="n"/>
+      <c r="H119" s="5" t="n"/>
+      <c r="I119" s="5" t="n"/>
+      <c r="J119" s="5" t="n"/>
       <c r="K119" s="5" t="n"/>
       <c r="L119" s="5" t="n"/>
       <c r="M119" s="5" t="n">
-        <v>8009.21</v>
+        <v>9594.559999999999</v>
       </c>
       <c r="N119" s="3" t="inlineStr">
         <is>
@@ -4743,72 +4737,105 @@
     <row r="120">
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>House Mart  (churned 2026-04)</t>
-        </is>
-      </c>
-      <c r="C120" s="5" t="n">
-        <v>6750</v>
-      </c>
+          <t>Reetal  (churned 2026-06)</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="n"/>
       <c r="D120" s="5" t="n"/>
       <c r="E120" s="5" t="n"/>
       <c r="F120" s="5" t="n"/>
-      <c r="G120" s="5" t="n"/>
+      <c r="G120" s="5" t="n">
+        <v>4492.3</v>
+      </c>
       <c r="H120" s="5" t="n">
-        <v>8800.5</v>
-      </c>
-      <c r="I120" s="5" t="n"/>
-      <c r="J120" s="5" t="n"/>
+        <v>1033.1</v>
+      </c>
+      <c r="I120" s="5" t="n">
+        <v>1799.32</v>
+      </c>
+      <c r="J120" s="5" t="n">
+        <v>684.49</v>
+      </c>
       <c r="K120" s="5" t="n"/>
       <c r="L120" s="5" t="n"/>
       <c r="M120" s="5" t="n">
+        <v>8009.21</v>
+      </c>
+      <c r="N120" s="3" t="inlineStr">
+        <is>
+          <t>Wafeq invoice export</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>House Mart  (churned 2026-04)</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="n">
+        <v>6750</v>
+      </c>
+      <c r="D121" s="5" t="n"/>
+      <c r="E121" s="5" t="n"/>
+      <c r="F121" s="5" t="n"/>
+      <c r="G121" s="5" t="n"/>
+      <c r="H121" s="5" t="n">
+        <v>8800.5</v>
+      </c>
+      <c r="I121" s="5" t="n"/>
+      <c r="J121" s="5" t="n"/>
+      <c r="K121" s="5" t="n"/>
+      <c r="L121" s="5" t="n"/>
+      <c r="M121" s="5" t="n">
         <v>15550.5</v>
       </c>
-      <c r="N120" s="3" t="inlineStr">
+      <c r="N121" s="3" t="inlineStr">
         <is>
           <t>Wafeq invoice export</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="B121" s="6" t="inlineStr">
+    <row r="122">
+      <c r="B122" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C121" s="7" t="n">
+      <c r="C122" s="7" t="n">
         <v>31390.44</v>
       </c>
-      <c r="D121" s="7" t="n">
+      <c r="D122" s="7" t="n">
         <v>21947.73</v>
       </c>
-      <c r="E121" s="7" t="n">
+      <c r="E122" s="7" t="n">
         <v>26212.8</v>
       </c>
-      <c r="F121" s="7" t="n">
+      <c r="F122" s="7" t="n">
         <v>19517.67</v>
       </c>
-      <c r="G121" s="7" t="n">
+      <c r="G122" s="7" t="n">
         <v>27125.53</v>
       </c>
-      <c r="H121" s="7" t="n">
+      <c r="H122" s="7" t="n">
         <v>27486.22</v>
       </c>
-      <c r="I121" s="7" t="n">
+      <c r="I122" s="7" t="n">
         <v>21956.43</v>
       </c>
-      <c r="J121" s="7" t="n">
+      <c r="J122" s="7" t="n">
         <v>16243.45</v>
       </c>
-      <c r="K121" s="7" t="n">
+      <c r="K122" s="7" t="n">
         <v>7298.95</v>
       </c>
-      <c r="L121" s="7" t="n">
+      <c r="L122" s="7" t="n">
         <v>2680.88</v>
       </c>
-      <c r="M121" s="7" t="n">
+      <c r="M122" s="7" t="n">
         <v>201860.1</v>
       </c>
-      <c r="N121" s="3" t="inlineStr">
+      <c r="N122" s="3" t="inlineStr">
         <is>
           <t>Wafeq invoice export</t>
         </is>

</xml_diff>

<commit_message>
Weekly run 13 Sep: no billing change, map Namshi ahead of its first invoice
Wafeq re-pulled today: 164 invoices, identical to the 9 Sep state. Nothing
issued, paid or amended in four days, so billed (211,873.82), receivables
(66,929.14) and every total are unchanged.

A new billing item, عمولة مبيعات - نمشي, was created in Wafeq on 10 Sep with
no invoice against it yet. Namshi is added to CH_AR and the platform channel
maps so the first invoice classifies as a Namshi commission rather than
falling into Other.

Platform data still the 30 Aug pull (read layer needs re-authorising);
Salla export 30 Aug; closed-PO export 17 Aug. Verification: 120 client-month
cells and 220 nested cells, 0 mismatches; allocation preserved; TOTAL holds.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bb5MYX3TP7gHh1Nbcy8kyQ
</commit_message>
<xml_diff>
--- a/revenue-view/output/Nasam_Revenue_View.xlsx
+++ b/revenue-view/output/Nasam_Revenue_View.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Nasam Revenue View — run of 9 Sep 2026 · August monthly close</t>
+          <t>Nasam Revenue View — weekly run · 13 Sep 2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -510,7 +510,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Monthly close for August, off the accounting drop Tarik shared on 9 Sep (data to 8 Sep). The four August invoices drafted on 31 Aug are now issued, so 10,013.72 moves from the memo line into billed — Wadi Halfa's released invoice is 8.11, not 2,008.11, because the 2,000 monthly fee was dropped while the shipping disruption lasts. New sheet 4 Cost &amp; Break-even carries the expense side for the first time: salaries and bills against revenue, what was spent on clients' behalf, how the gap was funded, and receivables reconciled against the accountant's statement. Platform sales, purchase orders and Sonbol's from-integration figure are still the 30 Aug pull (the read layer is offline).</t>
+          <t>A quiet week: no invoice was issued, paid or changed since 9 Sep, so billed, receivables and every total are unchanged. Wafeq was re-pulled today and matches the 9 Sep state exactly. One forward signal: a new billing item, عمولة مبيعات - نمشي (Namshi sales commission), was created in Wafeq on 10 Sep — the channel is now mapped here so the first Namshi invoice classifies correctly instead of falling into Other. Platform sales, purchase orders and Sonbol's from-integration figure are still the 30 Aug pull; the platform read layer needs re-authorising.</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Wafeq API snapshot 9 Sep (164 invoices) · Wafeq accounting exports 8 Sep: purchase bills, journal entries, customer-balances statement · platform revenue + purchase orders pulled 30 Aug (not refreshed) · churned-brand snapshots 15 Aug · Salla Partners export 30 Aug (manual, 26 records) · rate card 17 Aug.</t>
+          <t>Wafeq API snapshot 13 Sep (164 invoices) · Wafeq accounting exports 8 Sep: purchase bills, journal entries, customer-balances statement · platform revenue + purchase orders pulled 30 Aug (14 days old) · churned-brand snapshots 15 Aug · Salla Partners export 30 Aug (14 days old — the four trials live then have all since expired) · closed-PO export 17 Aug · rate card 17 Aug.</t>
         </is>
       </c>
     </row>

</xml_diff>